<commit_message>
IDEFICS-3 updated version of the DPE and DD
</commit_message>
<xml_diff>
--- a/analyst/Tracy/rmonize/data_dictionary/DD_IDEFICS_TRACY.xlsx
+++ b/analyst/Tracy/rmonize/data_dictionary/DD_IDEFICS_TRACY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Tracy\rmonize\data_dictionary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9255ECC8-6916-43C8-9586-C996B86CBCA3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A893CAD-9B97-4521-B94C-3FB47154786E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="57">
   <si>
     <t>index</t>
   </si>
@@ -191,19 +191,7 @@
     <t>employment status of the second person filled in the questionnaire</t>
   </si>
   <si>
-    <t>Use of  vitamin/multivitamin supplements in the last 7 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no </t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes </t>
-  </si>
-  <si>
     <t xml:space="preserve">ID </t>
-  </si>
-  <si>
-    <t>MED_SUPPL</t>
   </si>
 </sst>
 </file>
@@ -636,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -663,7 +651,7 @@
         <v>10</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>7</v>
@@ -790,25 +778,14 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>56</v>
+        <v>48</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>49</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -820,7 +797,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -1191,47 +1168,25 @@
         <v>28</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B34" s="3">
+        <v>48</v>
+      </c>
+      <c r="B34" s="11">
+        <v>1</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="11">
         <v>0</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B35" s="3">
-        <v>1</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="11">
-        <v>1</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B37" s="11">
-        <v>0</v>
-      </c>
-      <c r="C37" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>51</v>
       </c>
     </row>

</xml_diff>